<commit_message>
Bảng kê giải ngân: A4 ngang, cột nội dung rộng; ước lượng chiều cao dòng chữ HOA
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E35Rv4dC73JM56xVohPzXJ
</commit_message>
<xml_diff>
--- a/mau_chuan/BANG_KE_USD.xlsx
+++ b/mau_chuan/BANG_KE_USD.xlsx
@@ -519,13 +519,13 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4.5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -549,7 +549,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="8" customHeight="1"/>
+    <row r="4" ht="6" customHeight="1"/>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
       </c>
     </row>
     <row r="7" ht="8" customHeight="1"/>
-    <row r="8" ht="44" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Stt</t>
@@ -602,7 +602,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>{{CT.STT}}</t>
@@ -639,7 +639,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Tổng cộng</t>
@@ -661,14 +661,14 @@
       <c r="G10" s="9" t="n"/>
     </row>
     <row r="11" ht="8" customHeight="1"/>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Bằng chữ (USD): {{BANG_KE.TONG_TIEN_BANG_CHU}}</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Quy đổi bằng chữ (VND): {{BANG_KE.TONG_TIEN_QUY_DOI_BANG_CHU}}</t>
@@ -716,7 +716,7 @@
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.55" right="0.45" top="0.7" bottom="0.7" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bộ mẫu chuẩn: UNC 2 liên/A4 dọc, HĐMB không kẻ khung 1 trang, HĐTD nguyên bản (lề ô bảng), Bảng kê cột rộng + ngắt trang tránh trang chữ ký trống
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E35Rv4dC73JM56xVohPzXJ
</commit_message>
<xml_diff>
--- a/mau_chuan/BANG_KE_USD.xlsx
+++ b/mau_chuan/BANG_KE_USD.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,10 @@
     <font>
       <name val="Times New Roman"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Times New Roman"/>
@@ -110,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -136,19 +140,22 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -520,12 +527,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -602,7 +609,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>{{CT.STT}}</t>
@@ -633,43 +640,43 @@
           <t>{{CT.SO_TIEN_QUY_DOI_VN}}</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>{{CT.NOI_DUNG}}</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Tổng cộng</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>{{BANG_KE.TONG_TIEN_VN}}</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>{{BANG_KE.TONG_TIEN_QUY_DOI_VN}}</t>
         </is>
       </c>
-      <c r="G10" s="9" t="n"/>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11" ht="8" customHeight="1"/>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Bằng chữ (USD): {{BANG_KE.TONG_TIEN_BANG_CHU}}</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Quy đổi bằng chữ (VND): {{BANG_KE.TONG_TIEN_QUY_DOI_BANG_CHU}}</t>
         </is>
@@ -677,24 +684,24 @@
     </row>
     <row r="14" ht="14" customHeight="1"/>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>KẾ TOÁN TRƯỞNG</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>NGÂN HÀNG</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ tên)</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>(Ký, đóng dấu)</t>
         </is>

</xml_diff>